<commit_message>
Restore original refs for INFINITY TH 50 and TR 30 head flaps
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/LPG-Deutschland-Catalogue.xlsx
+++ b/LPG-Deutschland-Catalogue.xlsx
@@ -538,7 +538,6 @@
           <t>60.95</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>Körper</t>
@@ -628,7 +627,6 @@
           <t>60.95</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>Körper</t>
@@ -718,7 +716,6 @@
           <t>60.95</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
           <t>Körper</t>
@@ -808,7 +805,6 @@
           <t>60.95</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
           <t>Körper</t>
@@ -898,7 +894,6 @@
           <t>60.95</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
           <t>Körper</t>
@@ -988,7 +983,6 @@
           <t>60.95</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
           <t>Körper</t>
@@ -1078,7 +1072,6 @@
           <t>31.6</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
           <t>Körper</t>
@@ -1121,7 +1114,6 @@
           <t>87.4</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
           <t>Körper</t>
@@ -1211,7 +1203,6 @@
           <t>43.7</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
           <t>Gesicht</t>
@@ -1301,7 +1292,6 @@
           <t>35.65</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
           <t>Gesicht</t>
@@ -1391,7 +1381,6 @@
           <t>43.7</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
           <t>Gesicht</t>
@@ -1481,7 +1470,6 @@
           <t>46</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
           <t>Gesicht</t>
@@ -1561,13 +1549,11 @@
           <t>professionnel</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
           <t>44.85</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
           <t>Gesicht</t>
@@ -1657,7 +1643,6 @@
           <t>81.65</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
           <t>Gesicht</t>
@@ -1747,7 +1732,6 @@
           <t>67.85</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
           <t>Gesicht</t>
@@ -1837,7 +1821,6 @@
           <t>109</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
           <t>Gesicht</t>
@@ -1927,7 +1910,6 @@
           <t>79.35</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
         <is>
           <t>Gesicht</t>
@@ -2017,7 +1999,6 @@
           <t>78.1</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr">
         <is>
           <t>Gesicht</t>
@@ -2107,7 +2088,6 @@
           <t>60.95</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
           <t>Gesicht</t>
@@ -2197,7 +2177,6 @@
           <t>63.25</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
         <is>
           <t>Gesicht</t>
@@ -2287,7 +2266,6 @@
           <t>54</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr">
         <is>
           <t>Gesicht</t>
@@ -2377,7 +2355,6 @@
           <t>82.8</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
           <t>Gesicht</t>
@@ -2467,7 +2444,6 @@
           <t>40</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
           <t>Gesicht</t>
@@ -2557,7 +2533,6 @@
           <t>40</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
           <t>Gesicht</t>
@@ -2647,7 +2622,6 @@
           <t>58.65</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
           <t>Gesicht</t>
@@ -2737,7 +2711,6 @@
           <t>46</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
           <t>Gesicht</t>
@@ -2827,7 +2800,6 @@
           <t>29.3</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
         <is>
           <t>Gesicht</t>
@@ -2860,7 +2832,6 @@
           <t>revente</t>
         </is>
       </c>
-      <c r="D55" t="inlineStr"/>
       <c r="E55" t="inlineStr">
         <is>
           <t>9.2</t>
@@ -2913,7 +2884,6 @@
           <t>87.5</t>
         </is>
       </c>
-      <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr">
         <is>
           <t>Gesicht</t>
@@ -3003,7 +2973,6 @@
           <t>23</t>
         </is>
       </c>
-      <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
           <t>Gesicht</t>
@@ -3093,7 +3062,6 @@
           <t>18.4</t>
         </is>
       </c>
-      <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
           <t>Gesicht</t>
@@ -3136,7 +3104,6 @@
           <t>123.7</t>
         </is>
       </c>
-      <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
         <is>
           <t>Gesicht</t>
@@ -3179,7 +3146,6 @@
           <t>103.5</t>
         </is>
       </c>
-      <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr">
         <is>
           <t>Gesicht</t>
@@ -3212,13 +3178,11 @@
           <t>professionnel</t>
         </is>
       </c>
-      <c r="D63" t="inlineStr"/>
       <c r="E63" t="inlineStr">
         <is>
           <t>104</t>
         </is>
       </c>
-      <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr">
         <is>
           <t>Gesicht</t>
@@ -3778,7 +3742,6 @@
           <t>16.1</t>
         </is>
       </c>
-      <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr">
         <is>
           <t>Material-Bedarf</t>
@@ -3821,7 +3784,6 @@
           <t>16.1</t>
         </is>
       </c>
-      <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr">
         <is>
           <t>Material-Bedarf</t>
@@ -3864,7 +3826,6 @@
           <t>16.1</t>
         </is>
       </c>
-      <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr">
         <is>
           <t>Material-Bedarf</t>
@@ -3907,7 +3868,6 @@
           <t>16.1</t>
         </is>
       </c>
-      <c r="F78" t="inlineStr"/>
       <c r="G78" t="inlineStr">
         <is>
           <t>Material-Bedarf</t>
@@ -3940,13 +3900,11 @@
           <t>professionnel</t>
         </is>
       </c>
-      <c r="D79" t="inlineStr"/>
       <c r="E79" t="inlineStr">
         <is>
           <t>15.5</t>
         </is>
       </c>
-      <c r="F79" t="inlineStr"/>
       <c r="G79" t="inlineStr">
         <is>
           <t>Material-Bedarf</t>
@@ -3979,13 +3937,11 @@
           <t>professionnel</t>
         </is>
       </c>
-      <c r="D80" t="inlineStr"/>
       <c r="E80" t="inlineStr">
         <is>
           <t>17.8</t>
         </is>
       </c>
-      <c r="F80" t="inlineStr"/>
       <c r="G80" t="inlineStr">
         <is>
           <t>Material-Bedarf</t>
@@ -4018,13 +3974,11 @@
           <t>professionnel</t>
         </is>
       </c>
-      <c r="D81" t="inlineStr"/>
       <c r="E81" t="inlineStr">
         <is>
           <t>59</t>
         </is>
       </c>
-      <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr">
         <is>
           <t>Material-Bedarf</t>
@@ -4067,7 +4021,6 @@
           <t>33</t>
         </is>
       </c>
-      <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr">
         <is>
           <t>Material-Bedarf</t>
@@ -4110,7 +4063,6 @@
           <t>18</t>
         </is>
       </c>
-      <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr">
         <is>
           <t>Material-Bedarf</t>
@@ -4153,7 +4105,6 @@
           <t>15</t>
         </is>
       </c>
-      <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr">
         <is>
           <t>Material-Bedarf</t>
@@ -4196,7 +4147,6 @@
           <t>71</t>
         </is>
       </c>
-      <c r="F85" t="inlineStr"/>
       <c r="G85" t="inlineStr">
         <is>
           <t>Textilien</t>
@@ -4239,7 +4189,6 @@
           <t>71</t>
         </is>
       </c>
-      <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr">
         <is>
           <t>Textilien</t>
@@ -4282,7 +4231,6 @@
           <t>71</t>
         </is>
       </c>
-      <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr">
         <is>
           <t>Textilien</t>
@@ -4325,7 +4273,6 @@
           <t>71</t>
         </is>
       </c>
-      <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr">
         <is>
           <t>Textilien</t>
@@ -4368,7 +4315,6 @@
           <t>71</t>
         </is>
       </c>
-      <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr">
         <is>
           <t>Textilien</t>
@@ -4411,7 +4357,6 @@
           <t>71</t>
         </is>
       </c>
-      <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr">
         <is>
           <t>Textilien</t>
@@ -4454,7 +4399,6 @@
           <t>71</t>
         </is>
       </c>
-      <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr">
         <is>
           <t>Textilien</t>
@@ -4497,7 +4441,6 @@
           <t>71</t>
         </is>
       </c>
-      <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr">
         <is>
           <t>Textilien</t>
@@ -4540,7 +4483,6 @@
           <t>32</t>
         </is>
       </c>
-      <c r="F93" t="inlineStr"/>
       <c r="G93" t="inlineStr">
         <is>
           <t>Textilien</t>
@@ -4583,7 +4525,6 @@
           <t>32</t>
         </is>
       </c>
-      <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr">
         <is>
           <t>Textilien</t>
@@ -4626,7 +4567,6 @@
           <t>32</t>
         </is>
       </c>
-      <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr">
         <is>
           <t>Textilien</t>
@@ -4669,7 +4609,6 @@
           <t>32</t>
         </is>
       </c>
-      <c r="F96" t="inlineStr"/>
       <c r="G96" t="inlineStr">
         <is>
           <t>Textilien</t>
@@ -4712,7 +4651,6 @@
           <t>70</t>
         </is>
       </c>
-      <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr">
         <is>
           <t>Textilien</t>
@@ -4755,7 +4693,6 @@
           <t>70</t>
         </is>
       </c>
-      <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr">
         <is>
           <t>Textilien</t>
@@ -4798,7 +4735,6 @@
           <t>70</t>
         </is>
       </c>
-      <c r="F99" t="inlineStr"/>
       <c r="G99" t="inlineStr">
         <is>
           <t>Textilien</t>
@@ -4831,13 +4767,11 @@
           <t>professionnel</t>
         </is>
       </c>
-      <c r="D100" t="inlineStr"/>
       <c r="E100" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr">
         <is>
           <t>Textilien</t>
@@ -4880,7 +4814,6 @@
           <t>58</t>
         </is>
       </c>
-      <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr">
         <is>
           <t>Textilien</t>
@@ -4923,7 +4856,6 @@
           <t>2</t>
         </is>
       </c>
-      <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
         <is>
           <t>Textilien</t>
@@ -4966,7 +4898,6 @@
           <t>3880</t>
         </is>
       </c>
-      <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr">
         <is>
           <t>Mobilier</t>
@@ -5009,7 +4940,6 @@
           <t>1900</t>
         </is>
       </c>
-      <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr">
         <is>
           <t>Mobilier</t>
@@ -5052,7 +4982,6 @@
           <t>730</t>
         </is>
       </c>
-      <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr">
         <is>
           <t>Mobilier</t>
@@ -5095,7 +5024,6 @@
           <t>1145</t>
         </is>
       </c>
-      <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr">
         <is>
           <t>Mobilier</t>
@@ -5136,7 +5064,6 @@
       <c r="E107" t="n">
         <v>17.8</v>
       </c>
-      <c r="F107" t="inlineStr"/>
       <c r="G107" t="inlineStr">
         <is>
           <t>Technik</t>
@@ -5177,7 +5104,6 @@
       <c r="E108" t="n">
         <v>16.2</v>
       </c>
-      <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr">
         <is>
           <t>Technik</t>
@@ -5218,7 +5144,6 @@
       <c r="E109" t="n">
         <v>13</v>
       </c>
-      <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr">
         <is>
           <t>Technik</t>
@@ -5259,7 +5184,6 @@
       <c r="E110" t="n">
         <v>5.25</v>
       </c>
-      <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr">
         <is>
           <t>Technik</t>
@@ -5279,7 +5203,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>102253801</t>
+          <t>102253800</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -5300,7 +5224,6 @@
       <c r="E111" t="n">
         <v>7.55</v>
       </c>
-      <c r="F111" t="inlineStr"/>
       <c r="G111" t="inlineStr">
         <is>
           <t>Technik</t>
@@ -5320,7 +5243,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>102254102</t>
+          <t>102254101</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -5341,7 +5264,6 @@
       <c r="E112" t="n">
         <v>6.1</v>
       </c>
-      <c r="F112" t="inlineStr"/>
       <c r="G112" t="inlineStr">
         <is>
           <t>Technik</t>
@@ -5382,7 +5304,6 @@
       <c r="E113" t="n">
         <v>14.4</v>
       </c>
-      <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr">
         <is>
           <t>Technik</t>

</xml_diff>